<commit_message>
fix(rules): reprice Circle of the Sea to match its own spell list (v0.348)
The bundle was charged 11 (9) where its seven paid grants - Fog Cloud, Gust of
Wind, Ray of Frost, Shatter, Thunderwave, Lightning Bolt, Water Breathing -
total 1+1+4+1+1+2+2 = 12, and 10 as origin.

Its list is exactly the shape of Aberrant Sorcery's (a cantrip plus two spells
each at 1st, 2nd and 3rd) and that one was already charged 12 (10), so this was
a 1 AP slip rather than a deliberate discount.

All 21 bundles now derive exactly from their own spell lists, so Appendix J no
longer carries an outlier note. Guide updated in the same change: the Sea row
and the Druid class summary (varies 5-11 -> varies 5-12). No testing/expected
update needed - no fixture prices this bundle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qqVHKVk8YDzkqek8Z7757
</commit_message>
<xml_diff>
--- a/docs/analysis/PACT-bundle-pricing.xlsx
+++ b/docs/analysis/PACT-bundle-pricing.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>v0.347</t>
+          <t>v0.348</t>
         </is>
       </c>
     </row>
@@ -762,14 +762,14 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>This reproduces 20 of the 21 stored prices exactly; Circle of the Sea is the single miss (charged</t>
+          <t>As of DATA.version v0.348 this reproduces ALL 21 stored prices exactly. Circle of the Sea used to be</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>11/9 where its seven paid grants total 12/10 - the same shape as Aberrant Sorcery, charged 12/10).</t>
+          <t>the one miss - charged 11/9 where its list totals 12/10 - and was repriced to 12/10 in that version.</t>
         </is>
       </c>
     </row>
@@ -9481,10 +9481,10 @@
         <v/>
       </c>
       <c r="G8" s="9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I8" s="8">
         <f>G8-E8</f>

</xml_diff>